<commit_message>
Day 5: Full Goibibo Train Selenium with Pytest
</commit_message>
<xml_diff>
--- a/Capstone_Goibibo_Flights/data/booking_data.xlsx
+++ b/Capstone_Goibibo_Flights/data/booking_data.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\priyanshu\Downloads\program\pycharm\wipro\Capstone_Goibibo_Flights\Capstone_Goibibo_Flights\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3693090C-2B38-476E-886C-2CEFF8A1DC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E01E38-30FD-423E-A8CD-63A3792FD26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8928" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrainData" sheetId="1" r:id="rId1"/>
     <sheet name="FilterPreferences" sheetId="2" r:id="rId2"/>
+    <sheet name="PassengerDetails" sheetId="3" r:id="rId3"/>
+    <sheet name="PaymentDetails" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Source</t>
   </si>
@@ -56,19 +58,73 @@
   </si>
   <si>
     <t>june</t>
+  </si>
+  <si>
+    <t>FullName</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>MealOption</t>
+  </si>
+  <si>
+    <t>Veg</t>
+  </si>
+  <si>
+    <t>ContactMobile</t>
+  </si>
+  <si>
+    <t>ContactEmail</t>
+  </si>
+  <si>
+    <t>somesome@gmail.com</t>
+  </si>
+  <si>
+    <t>CardNumber</t>
+  </si>
+  <si>
+    <t>ExpiryYear</t>
+  </si>
+  <si>
+    <t>CVV</t>
+  </si>
+  <si>
+    <t>1234567812345670</t>
+  </si>
+  <si>
+    <t>CardName</t>
+  </si>
+  <si>
+    <t>ExpiryMonth</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF6AAB73"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -91,8 +147,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,14 +433,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.44140625" customWidth="1"/>
     <col min="3" max="3" width="12.109375" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -395,7 +454,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -417,13 +476,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CCC0CF-07C3-406B-9328-3B21CD3B3D87}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.88671875" customWidth="1"/>
     <col min="2" max="2" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -431,7 +490,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -442,4 +501,112 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B4B1F3B-28FC-4E2D-B01C-32A84B8FBBFE}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12.21875" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <v>9019019015</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3315C238-AAAC-456A-ACB3-E53F1CF362A6}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2">
+        <v>2030</v>
+      </c>
+      <c r="D2">
+        <v>123</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day 6: FINAL Goibibo Train Selenium with Pytest
</commit_message>
<xml_diff>
--- a/Capstone_Goibibo_Flights/data/booking_data.xlsx
+++ b/Capstone_Goibibo_Flights/data/booking_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\priyanshu\Downloads\program\pycharm\wipro\Capstone_Goibibo_Flights\Capstone_Goibibo_Flights\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E01E38-30FD-423E-A8CD-63A3792FD26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A2DC7A-F965-494A-8697-C00FDB6A5F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8928" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TrainData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Source</t>
   </si>
@@ -51,12 +51,6 @@
     <t>2A</t>
   </si>
   <si>
-    <t>delhi</t>
-  </si>
-  <si>
-    <t>agra</t>
-  </si>
-  <si>
     <t>june</t>
   </si>
   <si>
@@ -106,13 +100,25 @@
   </si>
   <si>
     <t>ExpiryMonth</t>
+  </si>
+  <si>
+    <t>ANVT</t>
+  </si>
+  <si>
+    <t>AGC</t>
+  </si>
+  <si>
+    <t>IRCTCID</t>
+  </si>
+  <si>
+    <t>priyanshu4902</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,9 +128,9 @@
     </font>
     <font>
       <sz val="9.8000000000000007"/>
-      <color rgb="FF6AAB73"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -147,8 +153,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -433,14 +442,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
     <col min="2" max="2" width="11.44140625" customWidth="1"/>
     <col min="3" max="3" width="12.109375" customWidth="1"/>
     <col min="4" max="4" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -454,15 +464,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
       </c>
       <c r="D2">
         <v>26</v>
@@ -476,13 +486,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CCC0CF-07C3-406B-9328-3B21CD3B3D87}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" customWidth="1"/>
     <col min="2" max="2" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -490,7 +500,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -505,53 +515,60 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B4B1F3B-28FC-4E2D-B01C-32A84B8FBBFE}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.21875" customWidth="1"/>
     <col min="4" max="4" width="12.44140625" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" customWidth="1"/>
     <col min="6" max="6" width="23.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>11</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>13</v>
       </c>
       <c r="B2">
         <v>32</v>
       </c>
       <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
       </c>
       <c r="E2">
         <v>9019019015</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -563,7 +580,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3315C238-AAAC-456A-ACB3-E53F1CF362A6}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.21875" customWidth="1"/>
     <col min="2" max="2" width="14.109375" customWidth="1"/>
@@ -571,26 +588,26 @@
     <col min="5" max="5" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="B2">
         <v>12</v>
@@ -602,7 +619,7 @@
         <v>123</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>